<commit_message>
Adiciona dropdown de perfil de risco, colunas de projecao e grafico melhorado
</commit_message>
<xml_diff>
--- a/Simulador_FII.xlsx
+++ b/Simulador_FII.xlsx
@@ -2,34 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulador" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfis" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
+    <definedName name="aporte">Simulador!$D$11</definedName>
+    <definedName name="patrimonio">Simulador!$D$14</definedName>
+    <definedName name="qtd_anos">Simulador!$D$12</definedName>
+    <definedName name="rendimento_carteira">Simulador!$D$7</definedName>
     <definedName name="salario">Simulador!$D$6</definedName>
-    <definedName name="rendimento_carteira">Simulador!$D$7</definedName>
     <definedName name="sugestao_investimento">Simulador!$D$8</definedName>
-    <definedName name="aporte">Simulador!$D$11</definedName>
-    <definedName name="qtd_anos">Simulador!$D$12</definedName>
     <definedName name="taxa_mensal">Simulador!$D$13</definedName>
-    <definedName name="patrimonio">Simulador!$D$14</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="\R\$\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,42 +40,58 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="18"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00404040"/>
+      <color rgb="FF404040"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00375623"/>
+      <color rgb="FF375623"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <i val="1"/>
@@ -83,7 +99,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -92,17 +108,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5496"/>
+        <fgColor rgb="FF2E5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -112,11 +138,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="002E5496"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -126,33 +152,38 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <bottom style="thin">
         <color rgb="00BFBFBF"/>
       </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -202,10 +233,6 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -224,9 +251,32 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -302,6 +352,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -312,7 +363,8 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Evolução do Patrimônio (primeiros 60 meses)</a:t>
+              <a:rPr sz="1400" b="1"/>
+              <a:t>Evolução do Patrimônio, Investimento e Rendimento</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -326,16 +378,20 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Simulador'!C29</f>
+              <f>'Simulador'!C27</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="3"/>
             <spPr>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -344,14 +400,89 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Simulador'!$B$30:$B$89</f>
+              <f>'Simulador'!$B$28:$B$87</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Simulador'!$C$30:$C$89</f>
+              <f>'Simulador'!$C$28:$C$87</f>
             </numRef>
           </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Simulador'!D27</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="A6A6A6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="3"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Simulador'!$B$28:$B$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Simulador'!$D$28:$D$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Simulador'!E27</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="375623"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="3"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Simulador'!$B$28:$B$87</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Simulador'!$E$28:$E$87</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -361,6 +492,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -387,8 +519,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
@@ -398,17 +530,21 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Patrimônio (R$)</a:t>
+                  <a:t>Valor (R$)</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="R$ #,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -419,12 +555,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>10</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2880000"/>
+    <ext cx="16459200" cy="8229600"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -731,982 +867,1476 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E103"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A2:M104"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="6.5703125" customWidth="1" style="28" min="1" max="1"/>
+    <col width="40" customWidth="1" style="28" min="2" max="2"/>
+    <col width="52.5703125" customWidth="1" style="28" min="3" max="3"/>
+    <col width="30.5703125" customWidth="1" style="28" min="4" max="4"/>
+    <col hidden="1" width="15.140625" customWidth="1" style="28" min="5" max="5"/>
+    <col width="0.140625" customWidth="1" style="28" min="6" max="6"/>
+    <col width="28.7109375" customWidth="1" style="28" min="7" max="7"/>
+    <col width="29.5703125" customWidth="1" style="28" min="8" max="8"/>
+    <col width="49.140625" customWidth="1" style="28" min="9" max="9"/>
+    <col hidden="1" style="28" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="2" ht="33.95" customHeight="1" s="28">
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>SIMULADOR DE INVESTIMENTOS EM FUNDOS IMOBILIÁRIOS (FII)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
+    <row r="3" ht="20.1" customHeight="1" s="28">
+      <c r="B3" s="31" t="inlineStr">
         <is>
           <t>Ferramenta de apoio à decisão: patrimônio acumulado, dividendos mensais e alocação por perfil</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="3" t="inlineStr">
+    <row r="5" ht="15.75" customHeight="1" s="28">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>CONFIGURAÇÕES DO INVESTIDOR</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>2000</v>
+      <c r="D6" s="2" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Rendimento médio da carteira (dividendos)</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="3" t="n">
         <v>0.006</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Sugestão de investimento (30% do salário)</t>
         </is>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="4">
         <f>D6*30%</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="3" t="inlineStr">
+    <row r="10" ht="15.75" customHeight="1" s="28">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>PARÂMETROS DA SIMULAÇÃO</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Quanto investir por mês?</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>200</v>
+      <c r="D11" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Por quantos anos?</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Taxa de rendimento mensal (valorização)?</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="3" t="n">
         <v>0.01079</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Patrimônio acumulado</t>
         </is>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="4">
         <f>FV(taxa_mensal,qtd_anos*12,aporte*-1)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Dividendos mensais estimados</t>
         </is>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="4">
         <f>patrimonio*rendimento_carteira</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Total efetivamente investido</t>
         </is>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="7">
         <f>aporte*qtd_anos*12</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Rendimento (juros) acumulado</t>
         </is>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="7">
         <f>patrimonio-D16</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="19" ht="15.75" customHeight="1" s="28">
+      <c r="B19" s="29" t="inlineStr">
         <is>
           <t>CENÁRIOS - EVOLUÇÃO DO PATRIMÔNIO</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+    <row r="20" ht="16.5" customHeight="1" s="28">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Patrimônio</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Dividendo Mensal</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="n">
+      <c r="G20" s="29" t="inlineStr">
+        <is>
+          <t>PERFIL DE ALOCAÇÃO DA CARTEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30.75" customHeight="1" s="28">
+      <c r="A21" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Quanto em 2 anos?</t>
         </is>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="11">
         <f>FV($D$13,A21*12,$D$11*-1)</f>
         <v/>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="7">
         <f>C21*rendimento_carteira</f>
         <v/>
       </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Perfil de risco</t>
+        </is>
+      </c>
+      <c r="H21" s="33" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="n">
+      <c r="A22" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Quanto em 5 anos?</t>
         </is>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="14">
         <f>FV($D$13,A22*12,$D$11*-1)</f>
         <v/>
       </c>
-      <c r="D22" s="18">
+      <c r="D22" s="15">
         <f>C22*rendimento_carteira</f>
         <v/>
       </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>Valor a ser investido por mês</t>
+        </is>
+      </c>
+      <c r="H22" s="15">
+        <f>aporte</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n">
+      <c r="A23" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Quanto em 10 anos?</t>
         </is>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="11">
         <f>FV($D$13,A23*12,$D$11*-1)</f>
         <v/>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="7">
         <f>C23*rendimento_carteira</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="n">
+    <row r="24" ht="48.75" customHeight="1" s="28">
+      <c r="A24" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Quanto em 20 anos?</t>
         </is>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="14">
         <f>FV($D$13,A24*12,$D$11*-1)</f>
         <v/>
       </c>
-      <c r="D24" s="18">
+      <c r="D24" s="15">
         <f>C24*rendimento_carteira</f>
         <v/>
       </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Tipo de FII</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Percentual Sugerido</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Valor Mensal (R$)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Quanto em 30 anos?</t>
         </is>
       </c>
-      <c r="C25" s="14">
+      <c r="C25" s="11">
         <f>FV($D$13,A25*12,$D$11*-1)</f>
         <v/>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="7">
         <f>C25*rendimento_carteira</f>
         <v/>
       </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>PAPEL</t>
+        </is>
+      </c>
+      <c r="H25" s="19">
+        <f>VLOOKUP($H$21&amp;"-"&amp;G25,Perfis!$A:$D,4,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I25" s="15">
+        <f>H25*$H$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="28">
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>PROJEÇÃO MENSAL (para visualização gráfica)</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>TIJOLO</t>
+        </is>
+      </c>
+      <c r="H26" s="19">
+        <f>VLOOKUP($H$21&amp;"-"&amp;G26,Perfis!$A:$D,4,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I26" s="15">
+        <f>H26*$H$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Mês</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Patrimônio (R$)</t>
+        </is>
+      </c>
+      <c r="D27" s="34" t="inlineStr">
+        <is>
+          <t>Total Investido (R$)</t>
+        </is>
+      </c>
+      <c r="E27" s="34" t="inlineStr">
+        <is>
+          <t>Rendimento (R$)</t>
+        </is>
+      </c>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>HÍBRIDOS</t>
+        </is>
+      </c>
+      <c r="H27" s="19">
+        <f>VLOOKUP($H$21&amp;"-"&amp;G27,Perfis!$A:$D,4,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I27" s="15">
+        <f>H27*$H$22</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>PROJEÇÃO MENSAL (para visualização gráfica)</t>
-        </is>
+      <c r="B28" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="17">
+        <f>FV($D$13,B28,$D$11*-1)</f>
+        <v/>
+      </c>
+      <c r="D28" s="35">
+        <f>aporte*B28</f>
+        <v/>
+      </c>
+      <c r="E28" s="35">
+        <f>C28-D28</f>
+        <v/>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>FOFs</t>
+        </is>
+      </c>
+      <c r="H28" s="19">
+        <f>VLOOKUP($H$21&amp;"-"&amp;G28,Perfis!$A:$D,4,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I28" s="15">
+        <f>H28*$H$22</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>Mês</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="inlineStr">
-        <is>
-          <t>Patrimônio (R$)</t>
-        </is>
+      <c r="B29" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="17">
+        <f>FV($D$13,B29,$D$11*-1)</f>
+        <v/>
+      </c>
+      <c r="D29" s="35">
+        <f>aporte*B29</f>
+        <v/>
+      </c>
+      <c r="E29" s="35">
+        <f>C29-D29</f>
+        <v/>
+      </c>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>DESENVOLVIMENTO</t>
+        </is>
+      </c>
+      <c r="H29" s="19">
+        <f>VLOOKUP($H$21&amp;"-"&amp;G29,Perfis!$A:$D,4,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I29" s="15">
+        <f>H29*$H$22</f>
+        <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="20">
+      <c r="B30" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="17">
         <f>FV($D$13,B30,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D30" s="35">
+        <f>aporte*B30</f>
+        <v/>
+      </c>
+      <c r="E30" s="35">
+        <f>C30-D30</f>
+        <v/>
+      </c>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>HOTELARIAS</t>
+        </is>
+      </c>
+      <c r="H30" s="19">
+        <f>VLOOKUP($H$21&amp;"-"&amp;G30,Perfis!$A:$D,4,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I30" s="15">
+        <f>H30*$H$22</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
-      <c r="B31" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C31" s="20">
+      <c r="B31" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="17">
         <f>FV($D$13,B31,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D31" s="35">
+        <f>aporte*B31</f>
+        <v/>
+      </c>
+      <c r="E31" s="35">
+        <f>C31-D31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
-      <c r="B32" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="C32" s="20">
+      <c r="B32" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="17">
         <f>FV($D$13,B32,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D32" s="35">
+        <f>aporte*B32</f>
+        <v/>
+      </c>
+      <c r="E32" s="35">
+        <f>C32-D32</f>
+        <v/>
+      </c>
+      <c r="G32" s="36" t="inlineStr">
+        <is>
+          <t>Dica: altere os valores em azul para simular cenários e use o menu suspenso em 'Perfil de risco' (H21) para recalcular a alocação por tipo de FII.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="B33" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="C33" s="20">
+      <c r="B33" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C33" s="17">
         <f>FV($D$13,B33,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D33" s="35">
+        <f>aporte*B33</f>
+        <v/>
+      </c>
+      <c r="E33" s="35">
+        <f>C33-D33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
-      <c r="B34" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="C34" s="20">
+      <c r="B34" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C34" s="17">
         <f>FV($D$13,B34,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D34" s="35">
+        <f>aporte*B34</f>
+        <v/>
+      </c>
+      <c r="E34" s="35">
+        <f>C34-D34</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
-      <c r="B35" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="C35" s="20">
+      <c r="B35" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C35" s="17">
         <f>FV($D$13,B35,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D35" s="35">
+        <f>aporte*B35</f>
+        <v/>
+      </c>
+      <c r="E35" s="35">
+        <f>C35-D35</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
-      <c r="B36" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="C36" s="20">
+      <c r="B36" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="C36" s="17">
         <f>FV($D$13,B36,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D36" s="35">
+        <f>aporte*B36</f>
+        <v/>
+      </c>
+      <c r="E36" s="35">
+        <f>C36-D36</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
-      <c r="B37" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="C37" s="20">
+      <c r="B37" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="C37" s="17">
         <f>FV($D$13,B37,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D37" s="35">
+        <f>aporte*B37</f>
+        <v/>
+      </c>
+      <c r="E37" s="35">
+        <f>C37-D37</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
-      <c r="B38" s="15" t="n">
-        <v>9</v>
-      </c>
-      <c r="C38" s="20">
+      <c r="B38" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C38" s="17">
         <f>FV($D$13,B38,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D38" s="35">
+        <f>aporte*B38</f>
+        <v/>
+      </c>
+      <c r="E38" s="35">
+        <f>C38-D38</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="B39" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="C39" s="20">
+      <c r="B39" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="C39" s="17">
         <f>FV($D$13,B39,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D39" s="35">
+        <f>aporte*B39</f>
+        <v/>
+      </c>
+      <c r="E39" s="35">
+        <f>C39-D39</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
-      <c r="B40" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="C40" s="20">
+      <c r="B40" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="C40" s="17">
         <f>FV($D$13,B40,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D40" s="35">
+        <f>aporte*B40</f>
+        <v/>
+      </c>
+      <c r="E40" s="35">
+        <f>C40-D40</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
-      <c r="B41" s="15" t="n">
-        <v>12</v>
-      </c>
-      <c r="C41" s="20">
+      <c r="B41" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="C41" s="17">
         <f>FV($D$13,B41,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D41" s="35">
+        <f>aporte*B41</f>
+        <v/>
+      </c>
+      <c r="E41" s="35">
+        <f>C41-D41</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
-      <c r="B42" s="15" t="n">
-        <v>13</v>
-      </c>
-      <c r="C42" s="20">
+      <c r="B42" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="C42" s="17">
         <f>FV($D$13,B42,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D42" s="35">
+        <f>aporte*B42</f>
+        <v/>
+      </c>
+      <c r="E42" s="35">
+        <f>C42-D42</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
-      <c r="B43" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="C43" s="20">
+      <c r="B43" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="C43" s="17">
         <f>FV($D$13,B43,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D43" s="35">
+        <f>aporte*B43</f>
+        <v/>
+      </c>
+      <c r="E43" s="35">
+        <f>C43-D43</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
-      <c r="B44" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="C44" s="20">
+      <c r="B44" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="C44" s="17">
         <f>FV($D$13,B44,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D44" s="35">
+        <f>aporte*B44</f>
+        <v/>
+      </c>
+      <c r="E44" s="35">
+        <f>C44-D44</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
-      <c r="B45" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="C45" s="20">
+      <c r="B45" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="C45" s="17">
         <f>FV($D$13,B45,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D45" s="35">
+        <f>aporte*B45</f>
+        <v/>
+      </c>
+      <c r="E45" s="35">
+        <f>C45-D45</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
-      <c r="B46" s="15" t="n">
-        <v>17</v>
-      </c>
-      <c r="C46" s="20">
+      <c r="B46" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="C46" s="17">
         <f>FV($D$13,B46,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D46" s="35">
+        <f>aporte*B46</f>
+        <v/>
+      </c>
+      <c r="E46" s="35">
+        <f>C46-D46</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
-      <c r="B47" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="C47" s="20">
+      <c r="B47" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="C47" s="17">
         <f>FV($D$13,B47,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D47" s="35">
+        <f>aporte*B47</f>
+        <v/>
+      </c>
+      <c r="E47" s="35">
+        <f>C47-D47</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
-      <c r="B48" s="15" t="n">
-        <v>19</v>
-      </c>
-      <c r="C48" s="20">
+      <c r="B48" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="C48" s="17">
         <f>FV($D$13,B48,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D48" s="35">
+        <f>aporte*B48</f>
+        <v/>
+      </c>
+      <c r="E48" s="35">
+        <f>C48-D48</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
-      <c r="B49" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="C49" s="20">
+      <c r="B49" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="C49" s="17">
         <f>FV($D$13,B49,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D49" s="35">
+        <f>aporte*B49</f>
+        <v/>
+      </c>
+      <c r="E49" s="35">
+        <f>C49-D49</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
-      <c r="B50" s="15" t="n">
-        <v>21</v>
-      </c>
-      <c r="C50" s="20">
+      <c r="B50" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="C50" s="17">
         <f>FV($D$13,B50,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D50" s="35">
+        <f>aporte*B50</f>
+        <v/>
+      </c>
+      <c r="E50" s="35">
+        <f>C50-D50</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
-      <c r="B51" s="15" t="n">
-        <v>22</v>
-      </c>
-      <c r="C51" s="20">
+      <c r="B51" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="C51" s="17">
         <f>FV($D$13,B51,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D51" s="35">
+        <f>aporte*B51</f>
+        <v/>
+      </c>
+      <c r="E51" s="35">
+        <f>C51-D51</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
-      <c r="B52" s="15" t="n">
-        <v>23</v>
-      </c>
-      <c r="C52" s="20">
+      <c r="B52" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="C52" s="17">
         <f>FV($D$13,B52,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D52" s="35">
+        <f>aporte*B52</f>
+        <v/>
+      </c>
+      <c r="E52" s="35">
+        <f>C52-D52</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
-      <c r="B53" s="15" t="n">
-        <v>24</v>
-      </c>
-      <c r="C53" s="20">
+      <c r="B53" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="C53" s="17">
         <f>FV($D$13,B53,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D53" s="35">
+        <f>aporte*B53</f>
+        <v/>
+      </c>
+      <c r="E53" s="35">
+        <f>C53-D53</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
-      <c r="B54" s="15" t="n">
-        <v>25</v>
-      </c>
-      <c r="C54" s="20">
+      <c r="B54" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="C54" s="17">
         <f>FV($D$13,B54,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D54" s="35">
+        <f>aporte*B54</f>
+        <v/>
+      </c>
+      <c r="E54" s="35">
+        <f>C54-D54</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
-      <c r="B55" s="15" t="n">
-        <v>26</v>
-      </c>
-      <c r="C55" s="20">
+      <c r="B55" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="C55" s="17">
         <f>FV($D$13,B55,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D55" s="35">
+        <f>aporte*B55</f>
+        <v/>
+      </c>
+      <c r="E55" s="35">
+        <f>C55-D55</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
-      <c r="B56" s="15" t="n">
-        <v>27</v>
-      </c>
-      <c r="C56" s="20">
+      <c r="B56" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="C56" s="17">
         <f>FV($D$13,B56,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D56" s="35">
+        <f>aporte*B56</f>
+        <v/>
+      </c>
+      <c r="E56" s="35">
+        <f>C56-D56</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
-      <c r="B57" s="15" t="n">
-        <v>28</v>
-      </c>
-      <c r="C57" s="20">
+      <c r="B57" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="C57" s="17">
         <f>FV($D$13,B57,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D57" s="35">
+        <f>aporte*B57</f>
+        <v/>
+      </c>
+      <c r="E57" s="35">
+        <f>C57-D57</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
-      <c r="B58" s="15" t="n">
-        <v>29</v>
-      </c>
-      <c r="C58" s="20">
+      <c r="B58" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="C58" s="17">
         <f>FV($D$13,B58,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D58" s="35">
+        <f>aporte*B58</f>
+        <v/>
+      </c>
+      <c r="E58" s="35">
+        <f>C58-D58</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
-      <c r="B59" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="C59" s="20">
+      <c r="B59" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="C59" s="17">
         <f>FV($D$13,B59,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D59" s="35">
+        <f>aporte*B59</f>
+        <v/>
+      </c>
+      <c r="E59" s="35">
+        <f>C59-D59</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
-      <c r="B60" s="15" t="n">
-        <v>31</v>
-      </c>
-      <c r="C60" s="20">
+      <c r="B60" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="C60" s="17">
         <f>FV($D$13,B60,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D60" s="35">
+        <f>aporte*B60</f>
+        <v/>
+      </c>
+      <c r="E60" s="35">
+        <f>C60-D60</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
-      <c r="B61" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="C61" s="20">
+      <c r="B61" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="C61" s="17">
         <f>FV($D$13,B61,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D61" s="35">
+        <f>aporte*B61</f>
+        <v/>
+      </c>
+      <c r="E61" s="35">
+        <f>C61-D61</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
-      <c r="B62" s="15" t="n">
-        <v>33</v>
-      </c>
-      <c r="C62" s="20">
+      <c r="B62" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="C62" s="17">
         <f>FV($D$13,B62,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D62" s="35">
+        <f>aporte*B62</f>
+        <v/>
+      </c>
+      <c r="E62" s="35">
+        <f>C62-D62</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
-      <c r="B63" s="15" t="n">
-        <v>34</v>
-      </c>
-      <c r="C63" s="20">
+      <c r="B63" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="C63" s="17">
         <f>FV($D$13,B63,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D63" s="35">
+        <f>aporte*B63</f>
+        <v/>
+      </c>
+      <c r="E63" s="35">
+        <f>C63-D63</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
-      <c r="B64" s="15" t="n">
-        <v>35</v>
-      </c>
-      <c r="C64" s="20">
+      <c r="B64" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="C64" s="17">
         <f>FV($D$13,B64,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D64" s="35">
+        <f>aporte*B64</f>
+        <v/>
+      </c>
+      <c r="E64" s="35">
+        <f>C64-D64</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
-      <c r="B65" s="15" t="n">
-        <v>36</v>
-      </c>
-      <c r="C65" s="20">
+      <c r="B65" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="C65" s="17">
         <f>FV($D$13,B65,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D65" s="35">
+        <f>aporte*B65</f>
+        <v/>
+      </c>
+      <c r="E65" s="35">
+        <f>C65-D65</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
-      <c r="B66" s="15" t="n">
-        <v>37</v>
-      </c>
-      <c r="C66" s="20">
+      <c r="B66" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="C66" s="17">
         <f>FV($D$13,B66,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D66" s="35">
+        <f>aporte*B66</f>
+        <v/>
+      </c>
+      <c r="E66" s="35">
+        <f>C66-D66</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
-      <c r="B67" s="15" t="n">
-        <v>38</v>
-      </c>
-      <c r="C67" s="20">
+      <c r="B67" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="C67" s="17">
         <f>FV($D$13,B67,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D67" s="35">
+        <f>aporte*B67</f>
+        <v/>
+      </c>
+      <c r="E67" s="35">
+        <f>C67-D67</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
-      <c r="B68" s="15" t="n">
-        <v>39</v>
-      </c>
-      <c r="C68" s="20">
+      <c r="B68" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="C68" s="17">
         <f>FV($D$13,B68,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D68" s="35">
+        <f>aporte*B68</f>
+        <v/>
+      </c>
+      <c r="E68" s="35">
+        <f>C68-D68</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
-      <c r="B69" s="15" t="n">
-        <v>40</v>
-      </c>
-      <c r="C69" s="20">
+      <c r="B69" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="C69" s="17">
         <f>FV($D$13,B69,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D69" s="35">
+        <f>aporte*B69</f>
+        <v/>
+      </c>
+      <c r="E69" s="35">
+        <f>C69-D69</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
-      <c r="B70" s="15" t="n">
-        <v>41</v>
-      </c>
-      <c r="C70" s="20">
+      <c r="B70" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="C70" s="17">
         <f>FV($D$13,B70,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D70" s="35">
+        <f>aporte*B70</f>
+        <v/>
+      </c>
+      <c r="E70" s="35">
+        <f>C70-D70</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
-      <c r="B71" s="15" t="n">
-        <v>42</v>
-      </c>
-      <c r="C71" s="20">
+      <c r="B71" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="C71" s="17">
         <f>FV($D$13,B71,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D71" s="35">
+        <f>aporte*B71</f>
+        <v/>
+      </c>
+      <c r="E71" s="35">
+        <f>C71-D71</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
-      <c r="B72" s="15" t="n">
-        <v>43</v>
-      </c>
-      <c r="C72" s="20">
+      <c r="B72" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="C72" s="17">
         <f>FV($D$13,B72,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D72" s="35">
+        <f>aporte*B72</f>
+        <v/>
+      </c>
+      <c r="E72" s="35">
+        <f>C72-D72</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
-      <c r="B73" s="15" t="n">
-        <v>44</v>
-      </c>
-      <c r="C73" s="20">
+      <c r="B73" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="C73" s="17">
         <f>FV($D$13,B73,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D73" s="35">
+        <f>aporte*B73</f>
+        <v/>
+      </c>
+      <c r="E73" s="35">
+        <f>C73-D73</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
-      <c r="B74" s="15" t="n">
-        <v>45</v>
-      </c>
-      <c r="C74" s="20">
+      <c r="B74" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="C74" s="17">
         <f>FV($D$13,B74,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D74" s="35">
+        <f>aporte*B74</f>
+        <v/>
+      </c>
+      <c r="E74" s="35">
+        <f>C74-D74</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
-      <c r="B75" s="15" t="n">
-        <v>46</v>
-      </c>
-      <c r="C75" s="20">
+      <c r="B75" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="C75" s="17">
         <f>FV($D$13,B75,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D75" s="35">
+        <f>aporte*B75</f>
+        <v/>
+      </c>
+      <c r="E75" s="35">
+        <f>C75-D75</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
-      <c r="B76" s="15" t="n">
-        <v>47</v>
-      </c>
-      <c r="C76" s="20">
+      <c r="B76" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="C76" s="17">
         <f>FV($D$13,B76,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D76" s="35">
+        <f>aporte*B76</f>
+        <v/>
+      </c>
+      <c r="E76" s="35">
+        <f>C76-D76</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
-      <c r="B77" s="15" t="n">
-        <v>48</v>
-      </c>
-      <c r="C77" s="20">
+      <c r="B77" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="C77" s="17">
         <f>FV($D$13,B77,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D77" s="35">
+        <f>aporte*B77</f>
+        <v/>
+      </c>
+      <c r="E77" s="35">
+        <f>C77-D77</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
-      <c r="B78" s="15" t="n">
-        <v>49</v>
-      </c>
-      <c r="C78" s="20">
+      <c r="B78" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="C78" s="17">
         <f>FV($D$13,B78,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D78" s="35">
+        <f>aporte*B78</f>
+        <v/>
+      </c>
+      <c r="E78" s="35">
+        <f>C78-D78</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
-      <c r="B79" s="15" t="n">
-        <v>50</v>
-      </c>
-      <c r="C79" s="20">
+      <c r="B79" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="C79" s="17">
         <f>FV($D$13,B79,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D79" s="35">
+        <f>aporte*B79</f>
+        <v/>
+      </c>
+      <c r="E79" s="35">
+        <f>C79-D79</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
-      <c r="B80" s="15" t="n">
-        <v>51</v>
-      </c>
-      <c r="C80" s="20">
+      <c r="B80" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="C80" s="17">
         <f>FV($D$13,B80,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D80" s="35">
+        <f>aporte*B80</f>
+        <v/>
+      </c>
+      <c r="E80" s="35">
+        <f>C80-D80</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
-      <c r="B81" s="15" t="n">
-        <v>52</v>
-      </c>
-      <c r="C81" s="20">
+      <c r="B81" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="C81" s="17">
         <f>FV($D$13,B81,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D81" s="35">
+        <f>aporte*B81</f>
+        <v/>
+      </c>
+      <c r="E81" s="35">
+        <f>C81-D81</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
-      <c r="B82" s="15" t="n">
-        <v>53</v>
-      </c>
-      <c r="C82" s="20">
+      <c r="B82" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="C82" s="17">
         <f>FV($D$13,B82,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D82" s="35">
+        <f>aporte*B82</f>
+        <v/>
+      </c>
+      <c r="E82" s="35">
+        <f>C82-D82</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
-      <c r="B83" s="15" t="n">
-        <v>54</v>
-      </c>
-      <c r="C83" s="20">
+      <c r="B83" s="12" t="n">
+        <v>56</v>
+      </c>
+      <c r="C83" s="17">
         <f>FV($D$13,B83,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D83" s="35">
+        <f>aporte*B83</f>
+        <v/>
+      </c>
+      <c r="E83" s="35">
+        <f>C83-D83</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
-      <c r="B84" s="15" t="n">
-        <v>55</v>
-      </c>
-      <c r="C84" s="20">
+      <c r="B84" s="12" t="n">
+        <v>57</v>
+      </c>
+      <c r="C84" s="17">
         <f>FV($D$13,B84,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D84" s="35">
+        <f>aporte*B84</f>
+        <v/>
+      </c>
+      <c r="E84" s="35">
+        <f>C84-D84</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
-      <c r="B85" s="15" t="n">
-        <v>56</v>
-      </c>
-      <c r="C85" s="20">
+      <c r="B85" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="C85" s="17">
         <f>FV($D$13,B85,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D85" s="35">
+        <f>aporte*B85</f>
+        <v/>
+      </c>
+      <c r="E85" s="35">
+        <f>C85-D85</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
-      <c r="B86" s="15" t="n">
-        <v>57</v>
-      </c>
-      <c r="C86" s="20">
+      <c r="B86" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="C86" s="17">
         <f>FV($D$13,B86,$D$11*-1)</f>
         <v/>
       </c>
+      <c r="D86" s="35">
+        <f>aporte*B86</f>
+        <v/>
+      </c>
+      <c r="E86" s="35">
+        <f>C86-D86</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
-      <c r="B87" s="15" t="n">
-        <v>58</v>
-      </c>
-      <c r="C87" s="20">
+      <c r="B87" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="C87" s="17">
         <f>FV($D$13,B87,$D$11*-1)</f>
         <v/>
       </c>
-    </row>
-    <row r="88">
-      <c r="B88" s="15" t="n">
-        <v>59</v>
-      </c>
-      <c r="C88" s="20">
-        <f>FV($D$13,B88,$D$11*-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="15" t="n">
-        <v>60</v>
-      </c>
-      <c r="C89" s="20">
-        <f>FV($D$13,B89,$D$11*-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>PERFIL DE ALOCAÇÃO DA CARTEIRA</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" s="8" t="inlineStr">
-        <is>
-          <t>Perfil de risco</t>
-        </is>
-      </c>
-      <c r="C92" s="21" t="inlineStr">
-        <is>
-          <t>Moderado</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>Valor a ser investido por mês</t>
-        </is>
-      </c>
-      <c r="C93" s="18">
-        <f>aporte</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="B95" s="11" t="inlineStr">
-        <is>
-          <t>Tipo de FII</t>
-        </is>
-      </c>
-      <c r="C95" s="11" t="inlineStr">
-        <is>
-          <t>Percentual Sugerido</t>
-        </is>
-      </c>
-      <c r="D95" s="11" t="inlineStr">
-        <is>
-          <t>Valor Mensal (R$)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="B96" s="16" t="inlineStr">
-        <is>
-          <t>PAPEL</t>
-        </is>
-      </c>
-      <c r="C96" s="22">
-        <f>VLOOKUP($C$92&amp;"-"&amp;B96,Perfis!$A:$D,4,FALSE)</f>
-        <v/>
-      </c>
-      <c r="D96" s="18">
-        <f>C96*$C$93</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97">
-      <c r="B97" s="16" t="inlineStr">
-        <is>
-          <t>TIJOLO</t>
-        </is>
-      </c>
-      <c r="C97" s="22">
-        <f>VLOOKUP($C$92&amp;"-"&amp;B97,Perfis!$A:$D,4,FALSE)</f>
-        <v/>
-      </c>
-      <c r="D97" s="18">
-        <f>C97*$C$93</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="B98" s="16" t="inlineStr">
-        <is>
-          <t>HÍBRIDOS</t>
-        </is>
-      </c>
-      <c r="C98" s="22">
-        <f>VLOOKUP($C$92&amp;"-"&amp;B98,Perfis!$A:$D,4,FALSE)</f>
-        <v/>
-      </c>
-      <c r="D98" s="18">
-        <f>C98*$C$93</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="B99" s="16" t="inlineStr">
-        <is>
-          <t>FOFs</t>
-        </is>
-      </c>
-      <c r="C99" s="22">
-        <f>VLOOKUP($C$92&amp;"-"&amp;B99,Perfis!$A:$D,4,FALSE)</f>
-        <v/>
-      </c>
-      <c r="D99" s="18">
-        <f>C99*$C$93</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100">
-      <c r="B100" s="16" t="inlineStr">
-        <is>
-          <t>DESENVOLVIMENTO</t>
-        </is>
-      </c>
-      <c r="C100" s="22">
-        <f>VLOOKUP($C$92&amp;"-"&amp;B100,Perfis!$A:$D,4,FALSE)</f>
-        <v/>
-      </c>
-      <c r="D100" s="18">
-        <f>C100*$C$93</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="B101" s="16" t="inlineStr">
-        <is>
-          <t>HOTELARIAS</t>
-        </is>
-      </c>
-      <c r="C101" s="22">
-        <f>VLOOKUP($C$92&amp;"-"&amp;B101,Perfis!$A:$D,4,FALSE)</f>
-        <v/>
-      </c>
-      <c r="D101" s="18">
-        <f>C101*$C$93</f>
-        <v/>
-      </c>
-    </row>
-    <row r="103">
-      <c r="B103" s="23" t="inlineStr">
-        <is>
-          <t>Dica: altere os valores em azul para simular diferentes cenários. Os campos verdes são calculados automaticamente.</t>
-        </is>
-      </c>
-    </row>
+      <c r="D87" s="35">
+        <f>aporte*B87</f>
+        <v/>
+      </c>
+      <c r="E87" s="35">
+        <f>C87-D87</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="G20:J20"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B2:E2"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B2:E2"/>
     <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="G32:J32"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Perfil inválido" error="Escolha um perfil: Conservador, Moderado ou Agressivo." promptTitle="Perfil de Risco" prompt="Selecione o perfil de risco da carteira." type="list">
+      <formula1>"Conservador,Moderado,Agressivo"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1721,385 +2351,330 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" style="28" min="1" max="1"/>
+    <col width="18" customWidth="1" style="28" min="2" max="3"/>
+    <col width="12" customWidth="1" style="28" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+    <row r="1" ht="26.1" customHeight="1" s="28">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>TABELA DE PERFIS E ALOCAÇÃO POR TIPO DE FII</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+    <row r="2" ht="15.75" customHeight="1" s="28">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>CHAVE</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>PERFIL</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>TIPO DE FII</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25">
-        <f>B3&amp;'-'&amp;C3</f>
-        <v/>
-      </c>
-      <c r="B3" s="25" t="inlineStr">
+      <c r="A3" s="20" t="n"/>
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C3" s="26" t="inlineStr">
+      <c r="C3" s="21" t="inlineStr">
         <is>
           <t>PAPEL</t>
         </is>
       </c>
-      <c r="D3" s="27" t="n">
+      <c r="D3" s="22" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28">
-        <f>B4&amp;'-'&amp;C4</f>
-        <v/>
-      </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>TIJOLO</t>
         </is>
       </c>
-      <c r="D4" s="30" t="n">
+      <c r="D4" s="25" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25">
-        <f>B5&amp;'-'&amp;C5</f>
-        <v/>
-      </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="A5" s="20" t="n"/>
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>HÍBRIDOS</t>
         </is>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="22" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28">
-        <f>B6&amp;'-'&amp;C6</f>
-        <v/>
-      </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>FOFs</t>
         </is>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="25" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25">
-        <f>B7&amp;'-'&amp;C7</f>
-        <v/>
-      </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="A7" s="20" t="n"/>
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>DESENVOLVIMENTO</t>
         </is>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28">
-        <f>B8&amp;'-'&amp;C8</f>
-        <v/>
-      </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>HOTELARIAS</t>
         </is>
       </c>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25">
-        <f>B9&amp;'-'&amp;C9</f>
-        <v/>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="A9" s="20" t="n"/>
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>PAPEL</t>
         </is>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="22" t="n">
         <v>0.32</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28">
-        <f>B10&amp;'-'&amp;C10</f>
-        <v/>
-      </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>TIJOLO</t>
         </is>
       </c>
-      <c r="D10" s="30" t="n">
+      <c r="D10" s="25" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25">
-        <f>B11&amp;'-'&amp;C11</f>
-        <v/>
-      </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="A11" s="20" t="n"/>
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>HÍBRIDOS</t>
         </is>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="22" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28">
-        <f>B12&amp;'-'&amp;C12</f>
-        <v/>
-      </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>FOFs</t>
         </is>
       </c>
-      <c r="D12" s="30" t="n">
+      <c r="D12" s="25" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25">
-        <f>B13&amp;'-'&amp;C13</f>
-        <v/>
-      </c>
-      <c r="B13" s="25" t="inlineStr">
+      <c r="A13" s="20" t="n"/>
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>DESENVOLVIMENTO</t>
         </is>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="22" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28">
-        <f>B14&amp;'-'&amp;C14</f>
-        <v/>
-      </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>HOTELARIAS</t>
         </is>
       </c>
-      <c r="D14" s="30" t="n">
+      <c r="D14" s="25" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25">
-        <f>B15&amp;'-'&amp;C15</f>
-        <v/>
-      </c>
-      <c r="B15" s="25" t="inlineStr">
+      <c r="A15" s="20" t="n"/>
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>PAPEL</t>
         </is>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="22" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28">
-        <f>B16&amp;'-'&amp;C16</f>
-        <v/>
-      </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C16" s="29" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>TIJOLO</t>
         </is>
       </c>
-      <c r="D16" s="30" t="n">
+      <c r="D16" s="25" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="25">
-        <f>B17&amp;'-'&amp;C17</f>
-        <v/>
-      </c>
-      <c r="B17" s="25" t="inlineStr">
+      <c r="A17" s="20" t="n"/>
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>HÍBRIDOS</t>
         </is>
       </c>
-      <c r="D17" s="27" t="n">
+      <c r="D17" s="22" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="28">
-        <f>B18&amp;'-'&amp;C18</f>
-        <v/>
-      </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C18" s="29" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>FOFs</t>
         </is>
       </c>
-      <c r="D18" s="30" t="n">
+      <c r="D18" s="25" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25">
-        <f>B19&amp;'-'&amp;C19</f>
-        <v/>
-      </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="A19" s="20" t="n"/>
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>DESENVOLVIMENTO</t>
         </is>
       </c>
-      <c r="D19" s="27" t="n">
+      <c r="D19" s="22" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28">
-        <f>B20&amp;'-'&amp;C20</f>
-        <v/>
-      </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>HOTELARIAS</t>
         </is>
       </c>
-      <c r="D20" s="30" t="n">
+      <c r="D20" s="25" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>Os percentuais representam a sugestão de alocação do aporte mensal conforme o perfil de risco selecionado.</t>
         </is>

</xml_diff>